<commit_message>
fix: resolve dates before NTP and FA=FC issues
</commit_message>
<xml_diff>
--- a/output/schedule_service/generated_schedule_mdl_candidates_output_match_all_projects_section6_ntp2024-03-01.xlsx
+++ b/output/schedule_service/generated_schedule_mdl_candidates_output_match_all_projects_section6_ntp2024-03-01.xlsx
@@ -2532,17 +2532,17 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2023-12-02</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>2024-01-01</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
@@ -2968,17 +2968,17 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2023-12-02</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>2024-01-01</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -3582,17 +3582,17 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2024-06-07</t>
+          <t>2024-08-09</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>2024-07-19</t>
+          <t>2024-09-20</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -4442,17 +4442,17 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>2024-11-26</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>2024-11-05</t>
+          <t>2025-01-07</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>2024-12-17</t>
+          <t>2025-02-18</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
@@ -4539,7 +4539,7 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; Control</t>
+          <t>Instrumentation &amp; Control (BLOCK #2)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -4874,17 +4874,17 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2024-06-07</t>
+          <t>2024-08-09</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>2024-07-19</t>
+          <t>2024-09-20</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
@@ -5953,7 +5953,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -6041,7 +6041,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>1SF1265W62A18</t>
+          <t>3SF1265W62A18</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6051,47 +6051,47 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #11 &gt; GTG #11 Auxiliary System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #3 &gt; Gas Turbine &amp; Generator #31 &amp; #32 &gt; GTG #31 &gt; GTG #31 Auxiliary System</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2008-05-17</t>
+          <t>2008-07-16</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2008-05-21</t>
+          <t>2008-07-20</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>2025-12-28</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -9105,17 +9105,17 @@
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr">
         <is>
-          <t>2023-12-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>2024-01-30</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>2024-02-29</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="W80" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>1PF1265W42A03.4P</t>
+          <t>1PF1265W42A03P</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #12 &gt; GTG #12 Fuel Gas Supply System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #11 &gt; GTG #11 Fuel Gas Supply System</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>2008-01-31</t>
+          <t>2008-01-30</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9836,17 +9836,17 @@
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="inlineStr">
         <is>
-          <t>2023-12-16</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="W87" t="inlineStr">
@@ -10014,17 +10014,17 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>2PF6500W70A07P</t>
+          <t>1PF6500W70A07P</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>(STG #20 &amp; UST Shelter) P.O &amp; Procurement - Main TR</t>
+          <t>(STG #10 &amp; UST Shelter) P.O &amp; Procurement - Main TR</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #2 &gt; Steam Turbine &amp; Generator #20 &gt; STG Unit Step-up Transformer</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Steam Turbine &amp; Generator #10 &gt; STG Unit Step-up Transformer</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>2008-07-14</t>
+          <t>2008-06-22</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">

</xml_diff>

<commit_message>
fix: add score matrix to match rule semantic
</commit_message>
<xml_diff>
--- a/output/schedule_service/generated_schedule_mdl_candidates_output_match_all_projects_section6_ntp2024-03-01.xlsx
+++ b/output/schedule_service/generated_schedule_mdl_candidates_output_match_all_projects_section6_ntp2024-03-01.xlsx
@@ -439,7 +439,7 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="54" customWidth="1" min="13" max="13"/>
+    <col width="56" customWidth="1" min="13" max="13"/>
     <col width="70" customWidth="1" min="14" max="14"/>
     <col width="29" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
@@ -845,57 +845,57 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0PF3520W68A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>(Condensate Tank) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System &gt; Condensate System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2007-06-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2008-01-30</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -954,17 +954,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0EF3520W00A01</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>(FGSS) P&amp;ID &amp; System Design</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2007-09-20</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1180,57 +1180,57 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0PF3520W68A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>(Condensate Tank) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System &gt; Condensate System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2007-06-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2008-01-30</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1293,57 +1293,57 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0PF3520W68A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>(Condensate Tank) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System &gt; Condensate System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2007-06-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2008-01-30</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1406,57 +1406,57 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0PF3520W68A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>(Condensate Tank) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System &gt; Condensate System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2007-06-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2008-01-30</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1515,57 +1515,57 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1PF1255W70A01.1P</t>
+          <t>3CF1265W90A06</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>(GTG#12 Electrical) P.O &amp; Procurement</t>
+          <t>(Air&amp;Flue Gas System) Installation- I&amp;C</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #12 &gt; GTG #12 Electrical System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #3 &gt; Gas Turbine &amp; Generator #31 &amp; #32 &gt; GTG #31 &gt; GTG #31 Air and Flue Gas System</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
+          <t>2008-07-02</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2008-03-31</t>
+          <t>2008-07-15</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2024-10-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1628,57 +1628,57 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0PF5000W36A03P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>(HVAC Equipment) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; HVAC &amp; Fire Fighting System &gt; HVAC System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2007-08-15</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2008-06-11</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2024-11-28</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2024-12-28</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1737,57 +1737,57 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1PF1265W42A12P</t>
+          <t>1CF1265W90A17.8</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>(Control Oil) P.O &amp; Procurement</t>
+          <t>(Control Oil) Installation- I&amp;C</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #11 &gt; GTG #11 Auxiliary System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #12 &gt; GTG #12 Auxiliary System</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
+          <t>2008-05-03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2008-01-31</t>
+          <t>2008-05-16</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2025-11-08</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2024-10-20</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1850,57 +1850,57 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0PF5000W36A03P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>(HVAC Equipment) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; HVAC &amp; Fire Fighting System &gt; HVAC System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2007-08-15</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2008-06-11</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2024-11-28</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2024-12-28</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -2072,57 +2072,57 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0PF5000W36A03P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>(HVAC Equipment) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; HVAC &amp; Fire Fighting System &gt; HVAC System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2007-08-15</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2008-06-11</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>2024-10-14</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2024-11-28</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2024-12-28</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1PF1265W42A12P</t>
+          <t>1SF1265W62A18</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>(Control Oil) P.O &amp; Procurement</t>
+          <t>(Control Oil) Loop chek</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2301,42 +2301,42 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
+          <t>2008-05-17</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2008-01-31</t>
+          <t>2008-05-21</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2024-06-27</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>2024-07-27</t>
+          <t>2025-10-13</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>2024-08-26</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2024-09-10</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2024-09-25</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -2395,57 +2395,57 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1PF2070W42A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>(STG #10 Aux. Equip) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Steam Turbine &amp; Generator #10 &gt; STG Auxiliary Equipment</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2007-04-30</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2008-07-31</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-09-18</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-10-18</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
+          <t>2024-11-17</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2024-12-02</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-12-17</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2025-02-16</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2605,57 +2605,57 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1PF2070W42A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>(STG #10 Aux. Equip) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Steam Turbine &amp; Generator #10 &gt; STG Auxiliary Equipment</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2007-04-30</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2008-07-31</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>2024-06-29</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2024-08-13</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>2024-08-28</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2024-09-12</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -3231,29 +3231,25 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1PF1265W42A12P</t>
+          <t>1EF6500W00A09</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>(Control Oil) P.O &amp; Procurement</t>
+          <t>(GTG #11 &amp; UAT Shelter) GA &amp; Load Data to Civil Design</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #11 &gt; GTG #11 Auxiliary System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Block #1 Early Power Block Common &gt; Electrical System &gt; Auxiliary Transformer</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>2008-01-31</t>
-        </is>
-      </c>
+          <t>2007-05-31</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
@@ -3429,57 +3425,57 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1PF1625W42A06.0P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>(HRSG #11 Main Stack) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; HRSG #11 &amp; #12 &gt; HRSG #11 &gt; Main Stack</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2007-06-04</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2008-01-31</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2024-07-04</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>2024-08-03</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2024-09-02</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2024-09-17</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
@@ -4067,57 +4063,57 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1PF2070W42A04P</t>
+          <t>1EF3030W00A01</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>(STG #10 Aux. Equip) P.O &amp; Procurement</t>
+          <t>(ACWS) P&amp;ID &amp; System Design</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Steam Turbine &amp; Generator #10 &gt; STG Auxiliary Equipment</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Block #1 Combined Power Block Common &gt; Auxiliary Cooling Water System</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2007-04-30</t>
+          <t>2007-04-02</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2008-07-31</t>
+          <t>2007-10-05</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>2024-08-11</t>
+          <t>2024-07-14</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>2024-09-10</t>
+          <t>2024-08-13</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>2024-09-12</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>2024-09-27</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2024-10-12</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>2024-11-24</t>
+          <t>2024-10-27</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
@@ -4180,12 +4176,12 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0PF4035W42A05.1P</t>
+          <t>0EF4035W16A02.1</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>(WWTS) P.O &amp; Procurement</t>
+          <t>(WWTS) Civil Design(incl. FDN)</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4200,7 +4196,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2008-09-01</t>
+          <t>2008-02-01</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4289,57 +4285,57 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1PF1255W70A01.1P</t>
+          <t>0EF3520W00A01</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>(GTG#12 Electrical) P.O &amp; Procurement</t>
+          <t>(FGSS) P&amp;ID &amp; System Design</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #12 &gt; GTG #12 Electrical System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2008-03-31</t>
+          <t>2007-09-20</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2024-08-20</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2024-09-19</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2024-10-19</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2024-10-20</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -5282,57 +5278,57 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>1PF2070W42A04P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>(STG #10 Aux. Equip) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Steam Turbine &amp; Generator #10 &gt; STG Auxiliary Equipment</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2007-04-30</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2008-07-31</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>2024-06-29</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2024-08-13</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>2024-08-28</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>2024-09-12</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -5391,27 +5387,27 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1CF1230W64A07.1</t>
+          <t>0EF3025W00A01.0</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>(Air Intake) Installation_Inlet Duct</t>
+          <t>(Intake Screening System) P&amp;ID &amp; System Design</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #12 &gt; GTG #12 Air Intake System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Intake Pump Structure</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2008-04-18</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2008-04-25</t>
+          <t>2007-10-29</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr"/>
@@ -5419,17 +5415,17 @@
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>2025-01-19</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2025-02-18</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -5492,12 +5488,12 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0PF4035W42A05.1P</t>
+          <t>0EF4035W16A02.1</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>(WWTS) P.O &amp; Procurement</t>
+          <t>(WWTS) Civil Design(incl. FDN)</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5512,7 +5508,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2008-09-01</t>
+          <t>2008-02-01</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -5710,17 +5706,17 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1PF3520W42A05.1P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>(Gas COMP PKG) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Block #1 Early Power Block Common &gt; Fuel Gas Supply System &gt; Gas Compressor</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -5730,7 +5726,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2008-04-14</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -6372,57 +6368,57 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>1PF1265W42A13P</t>
+          <t>0EF3520W00A01</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>(TCA Cooler) P.O &amp; Procurement</t>
+          <t>(FGSS) P&amp;ID &amp; System Design</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Power Plant Block #1 &gt; Gas Turbine &amp; Generator #11 &amp; #12 &gt; GTG #11 &gt; GTG #11 Fuel Gas Supply System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2007-03-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2008-02-29</t>
+          <t>2007-09-20</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2024-08-20</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>2024-09-05</t>
+          <t>2024-09-19</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2024-10-19</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>2024-10-20</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="W55" t="inlineStr">
@@ -6485,57 +6481,57 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>0PF6040W74A02.1P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>(Electrical Cable) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Electrical System &gt; Power &amp; Electrical Control Cables</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2007-09-19</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2008-03-25</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>2024-10-19</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>2024-12-18</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W56" t="inlineStr">
@@ -6594,12 +6590,12 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>1CF1255W70A05</t>
+          <t>1PF1255W70A01P</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>(GTG#11 Electrical) Installation- Protection Sys.</t>
+          <t>(GTG#11 Electrical) P.O &amp; Procurement</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -6609,42 +6605,42 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2008-08-01</t>
+          <t>2007-03-01</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2008-09-15</t>
+          <t>2008-03-31</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>2025-10-24</t>
+          <t>2024-05-23</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2024-06-22</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2024-07-22</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2024-08-06</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2024-08-21</t>
         </is>
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2024-09-05</t>
         </is>
       </c>
       <c r="W57" t="inlineStr">
@@ -7034,57 +7030,57 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>0PF6040W74A02.1P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>(Electrical Cable) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Electrical System &gt; Power &amp; Electrical Control Cables</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2007-09-19</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2008-03-25</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>2024-10-19</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>2024-12-18</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W61" t="inlineStr">
@@ -7353,57 +7349,57 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0PF6040W74A02.1P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>(Electrical Cable) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Electrical System &gt; Power &amp; Electrical Control Cables</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2007-09-19</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2008-03-25</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>2024-10-19</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>2024-12-18</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W64" t="inlineStr">
@@ -7575,17 +7571,17 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>0EF3520W00A02.2</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>(FOSS) P&amp;ID &amp; System Design</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Oil Supply System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -7595,7 +7591,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>2007-10-29</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -7785,57 +7781,57 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>0EF4035W00A01.1</t>
+          <t>0EF4035W16A02.2</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>(WWTS) P&amp;ID &amp; System Design</t>
+          <t>(WWT LEB) FDN Design</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Waste Water Treatment System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Waste Water Treatment System &gt; Waste Water Treatment LEB</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2007-04-02</t>
+          <t>2007-11-02</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>2007-12-07</t>
+          <t>2008-02-01</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>2024-05-02</t>
+          <t>2024-12-02</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2025-01-31</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
         <is>
-          <t>2024-07-16</t>
+          <t>2025-02-15</t>
         </is>
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2025-03-02</t>
         </is>
       </c>
       <c r="V68" t="inlineStr">
         <is>
-          <t>2024-08-15</t>
+          <t>2025-03-17</t>
         </is>
       </c>
       <c r="W68" t="inlineStr">
@@ -8011,12 +8007,12 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>0EF5534W32A04</t>
+          <t>0EF5534W16A02</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>(DWP BLDG) Structure Design</t>
+          <t>(DWP BLDG) FDN Design</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -8419,57 +8415,57 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>0PF3510W42A06P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>(COMP Air PKG) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Compressed Air System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2007-08-01</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>2008-04-30</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>2025-01-06</t>
+          <t>2024-08-20</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>2025-02-05</t>
+          <t>2024-09-19</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2024-10-19</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>2025-03-22</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2025-04-06</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>2025-04-21</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="W74" t="inlineStr">
@@ -8637,17 +8633,17 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>0PF3010W42A05P</t>
+          <t>0EF5534W16A02</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>(WTS) P.O &amp; Procurement</t>
+          <t>(DWP BLDG) FDN Design</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Water Treatment System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Water &amp; Air Supply System &gt; Water Treatment System &gt; Demi. Water Plant Building</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -8657,7 +8653,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>2008-09-01</t>
+          <t>2008-01-01</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8750,57 +8746,57 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>0PF3520W42A04.3P</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>(FOFP) P.O &amp; Procurement</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Oil Supply System &gt; Fuel Oil Forward Station</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2007-07-02</t>
+          <t>2007-03-15</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>2008-03-28</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>2024-08-01</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>2024-08-31</t>
+          <t>2024-05-14</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>2024-09-30</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
         <is>
-          <t>2024-10-15</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="U77" t="inlineStr">
         <is>
-          <t>2024-10-30</t>
+          <t>2024-07-13</t>
         </is>
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>2024-11-14</t>
+          <t>2024-07-28</t>
         </is>
       </c>
       <c r="W77" t="inlineStr">
@@ -8968,17 +8964,17 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>0EF3520W00A01</t>
+          <t>0EF1000W00A04</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>(FGSS) P&amp;ID &amp; System Design</t>
+          <t>Mechanical Design Criteria</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant Common &gt; Fuel Gas &amp; Oil Supply Systems &gt; Fuel Gas Supply System</t>
+          <t>CCPP Project Standard Schedule_20181012_Idea &gt; Plant General &gt; Plant Engineering &gt; Basic Engineering &amp; Design</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -8988,7 +8984,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>2007-09-20</t>
+          <t>2007-07-24</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">

</xml_diff>